<commit_message>
fnew files should run now, and images updated
</commit_message>
<xml_diff>
--- a/Output Files GPT-OSS 20B/rag_ablation_results.xlsx
+++ b/Output Files GPT-OSS 20B/rag_ablation_results.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AS10"/>
+  <dimension ref="A1:AS7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -646,12 +646,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>nearest_neighbor_k3</t>
+          <t>control_k3</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Nearest-neighbor prediction k=3</t>
+          <t>Control k=3 standard</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -701,7 +701,7 @@
         <v>1</v>
       </c>
       <c r="O2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P2" t="inlineStr">
         <is>
@@ -709,22 +709,22 @@
         </is>
       </c>
       <c r="Q2" t="n">
-        <v>6.704444444444444</v>
+        <v>0.4</v>
       </c>
       <c r="R2" t="n">
-        <v>6.745555555555555</v>
+        <v>0.4</v>
       </c>
       <c r="S2" t="n">
-        <v>7.58</v>
+        <v>0.6</v>
       </c>
       <c r="T2" t="n">
-        <v>7.857777777777778</v>
+        <v>0.8</v>
       </c>
       <c r="U2" t="n">
-        <v>7.066944444444443</v>
+        <v>0.5</v>
       </c>
       <c r="V2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="W2" t="n">
         <v>4.491</v>
@@ -739,19 +739,19 @@
         <v>3</v>
       </c>
       <c r="AA2" t="n">
-        <v>2.12787962962963</v>
+        <v>4.694499999999999</v>
       </c>
       <c r="AB2" t="n">
-        <v>2.183026472227605</v>
+        <v>4.72317884656792</v>
       </c>
       <c r="AC2" t="n">
-        <v>0.816496580927726</v>
+        <v>0.3333333333333334</v>
       </c>
       <c r="AD2" t="n">
-        <v>0.8660254037844387</v>
+        <v>0.5</v>
       </c>
       <c r="AE2" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AF2" t="b">
         <v>1</v>
@@ -763,48 +763,50 @@
       </c>
       <c r="AH2" t="inlineStr">
         <is>
-          <t>68</t>
+          <t>64</t>
         </is>
       </c>
       <c r="AI2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AJ2" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AK2" t="n">
         <v>0</v>
       </c>
       <c r="AL2" t="n">
-        <v>0</v>
+        <v>3636</v>
       </c>
       <c r="AM2" t="n">
-        <v>0</v>
+        <v>398</v>
       </c>
       <c r="AN2" t="n">
-        <v>0</v>
+        <v>4034</v>
       </c>
       <c r="AO2" t="n">
-        <v>0</v>
+        <v>3029.376029968262</v>
       </c>
       <c r="AP2" t="inlineStr"/>
       <c r="AQ2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AR2" t="n">
         <v>1</v>
       </c>
-      <c r="AS2" t="inlineStr"/>
+      <c r="AS2" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>nearest_neighbor_k3</t>
+          <t>control_k3</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Nearest-neighbor prediction k=3</t>
+          <t>Control k=3 standard</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -854,7 +856,7 @@
         <v>1</v>
       </c>
       <c r="O3" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P3" t="inlineStr">
         <is>
@@ -862,22 +864,22 @@
         </is>
       </c>
       <c r="Q3" t="n">
-        <v>6.704444444444444</v>
+        <v>0.8</v>
       </c>
       <c r="R3" t="n">
-        <v>6.745555555555555</v>
+        <v>0.8</v>
       </c>
       <c r="S3" t="n">
-        <v>7.58</v>
+        <v>0.5</v>
       </c>
       <c r="T3" t="n">
-        <v>7.857777777777778</v>
+        <v>0.9</v>
       </c>
       <c r="U3" t="n">
-        <v>7.066944444444443</v>
+        <v>0.755</v>
       </c>
       <c r="V3" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="W3" t="n">
         <v>5.616999999999999</v>
@@ -892,19 +894,19 @@
         <v>3</v>
       </c>
       <c r="AA3" t="n">
-        <v>2.12787962962963</v>
+        <v>4.694499999999999</v>
       </c>
       <c r="AB3" t="n">
-        <v>2.183026472227605</v>
+        <v>4.72317884656792</v>
       </c>
       <c r="AC3" t="n">
-        <v>0.816496580927726</v>
+        <v>0.3333333333333334</v>
       </c>
       <c r="AD3" t="n">
-        <v>0.8660254037844387</v>
+        <v>0.5</v>
       </c>
       <c r="AE3" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AF3" t="b">
         <v>1</v>
@@ -916,48 +918,50 @@
       </c>
       <c r="AH3" t="inlineStr">
         <is>
-          <t>68</t>
+          <t>64</t>
         </is>
       </c>
       <c r="AI3" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AJ3" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AK3" t="n">
         <v>0</v>
       </c>
       <c r="AL3" t="n">
-        <v>0</v>
+        <v>3636</v>
       </c>
       <c r="AM3" t="n">
-        <v>0</v>
+        <v>398</v>
       </c>
       <c r="AN3" t="n">
-        <v>0</v>
+        <v>4034</v>
       </c>
       <c r="AO3" t="n">
-        <v>0</v>
+        <v>3029.376029968262</v>
       </c>
       <c r="AP3" t="inlineStr"/>
       <c r="AQ3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AR3" t="n">
         <v>1</v>
       </c>
-      <c r="AS3" t="inlineStr"/>
+      <c r="AS3" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>nearest_neighbor_k3</t>
+          <t>control_k3</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Nearest-neighbor prediction k=3</t>
+          <t>Control k=3 standard</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -1007,7 +1011,7 @@
         <v>1</v>
       </c>
       <c r="O4" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P4" t="inlineStr">
         <is>
@@ -1015,22 +1019,22 @@
         </is>
       </c>
       <c r="Q4" t="n">
-        <v>8.470000000000001</v>
+        <v>0.6</v>
       </c>
       <c r="R4" t="n">
-        <v>8.49</v>
+        <v>0.8</v>
       </c>
       <c r="S4" t="n">
-        <v>8.530000000000001</v>
+        <v>0.7</v>
       </c>
       <c r="T4" t="n">
-        <v>7.265000000000001</v>
+        <v>0.8</v>
       </c>
       <c r="U4" t="n">
-        <v>8.308250000000001</v>
+        <v>0.72</v>
       </c>
       <c r="V4" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="W4" t="n">
         <v>5.9505</v>
@@ -1045,19 +1049,19 @@
         <v>3</v>
       </c>
       <c r="AA4" t="n">
-        <v>2.12787962962963</v>
+        <v>4.694499999999999</v>
       </c>
       <c r="AB4" t="n">
-        <v>2.183026472227605</v>
+        <v>4.72317884656792</v>
       </c>
       <c r="AC4" t="n">
-        <v>0.816496580927726</v>
+        <v>0.3333333333333334</v>
       </c>
       <c r="AD4" t="n">
-        <v>0.8660254037844387</v>
+        <v>0.5</v>
       </c>
       <c r="AE4" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AF4" t="b">
         <v>1</v>
@@ -1069,48 +1073,50 @@
       </c>
       <c r="AH4" t="inlineStr">
         <is>
-          <t>68</t>
+          <t>64</t>
         </is>
       </c>
       <c r="AI4" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AJ4" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AK4" t="n">
         <v>0</v>
       </c>
       <c r="AL4" t="n">
-        <v>0</v>
+        <v>3636</v>
       </c>
       <c r="AM4" t="n">
-        <v>0</v>
+        <v>398</v>
       </c>
       <c r="AN4" t="n">
-        <v>0</v>
+        <v>4034</v>
       </c>
       <c r="AO4" t="n">
-        <v>0</v>
+        <v>3029.376029968262</v>
       </c>
       <c r="AP4" t="inlineStr"/>
       <c r="AQ4" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AR4" t="n">
         <v>1</v>
       </c>
-      <c r="AS4" t="inlineStr"/>
+      <c r="AS4" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>nearest_neighbor_k3</t>
+          <t>control_k3</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Nearest-neighbor prediction k=3</t>
+          <t>Control k=3 standard</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -1160,7 +1166,7 @@
         <v>1</v>
       </c>
       <c r="O5" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P5" t="inlineStr">
         <is>
@@ -1168,22 +1174,22 @@
         </is>
       </c>
       <c r="Q5" t="n">
-        <v>5.465555555555556</v>
+        <v>0.48</v>
       </c>
       <c r="R5" t="n">
-        <v>2.844444444444444</v>
+        <v>0.32</v>
       </c>
       <c r="S5" t="n">
-        <v>7.845555555555555</v>
+        <v>0.88</v>
       </c>
       <c r="T5" t="n">
-        <v>7.068888888888889</v>
+        <v>0.82</v>
       </c>
       <c r="U5" t="n">
-        <v>5.264666666666667</v>
+        <v>0.5549999999999999</v>
       </c>
       <c r="V5" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="W5" t="n">
         <v>6.013</v>
@@ -1198,19 +1204,19 @@
         <v>3</v>
       </c>
       <c r="AA5" t="n">
-        <v>1.478833333333333</v>
+        <v>3.456166666666667</v>
       </c>
       <c r="AB5" t="n">
-        <v>1.58176292003106</v>
+        <v>3.759719858801539</v>
       </c>
       <c r="AC5" t="n">
-        <v>0.816496580927726</v>
+        <v>0.3333333333333334</v>
       </c>
       <c r="AD5" t="n">
-        <v>0.8660254037844387</v>
+        <v>0.5</v>
       </c>
       <c r="AE5" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AF5" t="b">
         <v>1</v>
@@ -1222,48 +1228,50 @@
       </c>
       <c r="AH5" t="inlineStr">
         <is>
-          <t>8:00 AM</t>
+          <t>11:00 PM</t>
         </is>
       </c>
       <c r="AI5" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AJ5" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AK5" t="n">
         <v>0</v>
       </c>
       <c r="AL5" t="n">
-        <v>0</v>
+        <v>3507</v>
       </c>
       <c r="AM5" t="n">
-        <v>0</v>
+        <v>472</v>
       </c>
       <c r="AN5" t="n">
-        <v>0</v>
+        <v>3979</v>
       </c>
       <c r="AO5" t="n">
-        <v>0</v>
+        <v>3132.863521575928</v>
       </c>
       <c r="AP5" t="inlineStr"/>
       <c r="AQ5" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AR5" t="n">
         <v>1</v>
       </c>
-      <c r="AS5" t="inlineStr"/>
+      <c r="AS5" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>nearest_neighbor_k3</t>
+          <t>control_k3</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Nearest-neighbor prediction k=3</t>
+          <t>Control k=3 standard</t>
         </is>
       </c>
       <c r="C6" t="n">
@@ -1313,7 +1321,7 @@
         <v>1</v>
       </c>
       <c r="O6" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P6" t="inlineStr">
         <is>
@@ -1321,19 +1329,19 @@
         </is>
       </c>
       <c r="Q6" t="n">
-        <v>2.96</v>
+        <v>0.5</v>
       </c>
       <c r="R6" t="n">
-        <v>3.1</v>
+        <v>0.5</v>
       </c>
       <c r="S6" t="n">
-        <v>7.81</v>
+        <v>0.4</v>
       </c>
       <c r="T6" t="n">
-        <v>6.66</v>
+        <v>0.6</v>
       </c>
       <c r="U6" t="n">
-        <v>4.534</v>
+        <v>0.495</v>
       </c>
       <c r="V6" t="n">
         <v>3</v>
@@ -1351,19 +1359,19 @@
         <v>3</v>
       </c>
       <c r="AA6" t="n">
-        <v>1.478833333333333</v>
+        <v>3.456166666666667</v>
       </c>
       <c r="AB6" t="n">
-        <v>1.58176292003106</v>
+        <v>3.759719858801539</v>
       </c>
       <c r="AC6" t="n">
-        <v>0.816496580927726</v>
+        <v>0.3333333333333334</v>
       </c>
       <c r="AD6" t="n">
-        <v>0.8660254037844387</v>
+        <v>0.5</v>
       </c>
       <c r="AE6" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AF6" t="b">
         <v>1</v>
@@ -1375,48 +1383,50 @@
       </c>
       <c r="AH6" t="inlineStr">
         <is>
-          <t>8:00 AM</t>
+          <t>11:00 PM</t>
         </is>
       </c>
       <c r="AI6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AJ6" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AK6" t="n">
         <v>0</v>
       </c>
       <c r="AL6" t="n">
-        <v>0</v>
+        <v>3507</v>
       </c>
       <c r="AM6" t="n">
-        <v>0</v>
+        <v>472</v>
       </c>
       <c r="AN6" t="n">
-        <v>0</v>
+        <v>3979</v>
       </c>
       <c r="AO6" t="n">
-        <v>0</v>
+        <v>3132.863521575928</v>
       </c>
       <c r="AP6" t="inlineStr"/>
       <c r="AQ6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AR6" t="n">
         <v>1</v>
       </c>
-      <c r="AS6" t="inlineStr"/>
+      <c r="AS6" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>nearest_neighbor_k3</t>
+          <t>control_k3</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Nearest-neighbor prediction k=3</t>
+          <t>Control k=3 standard</t>
         </is>
       </c>
       <c r="C7" t="n">
@@ -1466,7 +1476,7 @@
         <v>1</v>
       </c>
       <c r="O7" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P7" t="inlineStr">
         <is>
@@ -1474,22 +1484,22 @@
         </is>
       </c>
       <c r="Q7" t="n">
-        <v>5.465555555555556</v>
+        <v>0.9</v>
       </c>
       <c r="R7" t="n">
-        <v>2.844444444444444</v>
+        <v>0.9</v>
       </c>
       <c r="S7" t="n">
-        <v>7.845555555555555</v>
+        <v>0.3</v>
       </c>
       <c r="T7" t="n">
-        <v>7.068888888888889</v>
+        <v>0.4</v>
       </c>
       <c r="U7" t="n">
-        <v>5.264666666666667</v>
+        <v>0.7050000000000001</v>
       </c>
       <c r="V7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="W7" t="n">
         <v>3.6895</v>
@@ -1504,19 +1514,19 @@
         <v>3</v>
       </c>
       <c r="AA7" t="n">
-        <v>1.478833333333333</v>
+        <v>3.456166666666667</v>
       </c>
       <c r="AB7" t="n">
-        <v>1.58176292003106</v>
+        <v>3.759719858801539</v>
       </c>
       <c r="AC7" t="n">
-        <v>0.816496580927726</v>
+        <v>0.3333333333333334</v>
       </c>
       <c r="AD7" t="n">
-        <v>0.8660254037844387</v>
+        <v>0.5</v>
       </c>
       <c r="AE7" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AF7" t="b">
         <v>1</v>
@@ -1528,485 +1538,40 @@
       </c>
       <c r="AH7" t="inlineStr">
         <is>
-          <t>8:00 AM</t>
+          <t>11:00 PM</t>
         </is>
       </c>
       <c r="AI7" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AJ7" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AK7" t="n">
         <v>0</v>
       </c>
       <c r="AL7" t="n">
-        <v>0</v>
+        <v>3507</v>
       </c>
       <c r="AM7" t="n">
-        <v>0</v>
+        <v>472</v>
       </c>
       <c r="AN7" t="n">
-        <v>0</v>
+        <v>3979</v>
       </c>
       <c r="AO7" t="n">
-        <v>0</v>
+        <v>3132.863521575928</v>
       </c>
       <c r="AP7" t="inlineStr"/>
       <c r="AQ7" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="AR7" t="n">
         <v>1</v>
       </c>
-      <c r="AS7" t="inlineStr"/>
-    </row>
-    <row r="8">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>nearest_neighbor_k3</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>Nearest-neighbor prediction k=3</t>
-        </is>
-      </c>
-      <c r="C8" t="n">
-        <v>17</v>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>Shower</t>
-        </is>
-      </c>
-      <c r="E8" t="n">
-        <v>17</v>
-      </c>
-      <c r="F8" t="n">
-        <v>17</v>
-      </c>
-      <c r="G8" t="inlineStr">
-        <is>
-          <t>How long should I shower?</t>
-        </is>
-      </c>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>West Mifflin, PA</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>similarity</t>
-        </is>
-      </c>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>sentence-transformers/all-MiniLM-L6-v2</t>
-        </is>
-      </c>
-      <c r="K8" t="n">
-        <v>3</v>
-      </c>
-      <c r="L8" t="b">
-        <v>1</v>
-      </c>
-      <c r="M8" t="b">
-        <v>1</v>
-      </c>
-      <c r="N8" t="b">
-        <v>1</v>
-      </c>
-      <c r="O8" t="b">
-        <v>0</v>
-      </c>
-      <c r="P8" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="Q8" t="n">
-        <v>8.044444444444444</v>
-      </c>
-      <c r="R8" t="n">
-        <v>7.506666666666667</v>
-      </c>
-      <c r="S8" t="n">
-        <v>7.517777777777777</v>
-      </c>
-      <c r="T8" t="n">
-        <v>3.522222222222222</v>
-      </c>
-      <c r="U8" t="n">
-        <v>7.072555555555555</v>
-      </c>
-      <c r="V8" t="n">
-        <v>1</v>
-      </c>
-      <c r="W8" t="n">
-        <v>7.608999999999999</v>
-      </c>
-      <c r="X8" t="n">
-        <v>1</v>
-      </c>
-      <c r="Y8" t="n">
-        <v>0.04096141892174879</v>
-      </c>
-      <c r="Z8" t="n">
-        <v>3</v>
-      </c>
-      <c r="AA8" t="n">
-        <v>0.3688148148148149</v>
-      </c>
-      <c r="AB8" t="n">
-        <v>0.3875168733881066</v>
-      </c>
-      <c r="AC8" t="inlineStr"/>
-      <c r="AD8" t="inlineStr"/>
-      <c r="AE8" t="b">
-        <v>1</v>
-      </c>
-      <c r="AF8" t="b">
-        <v>1</v>
-      </c>
-      <c r="AG8" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="AH8" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="AI8" t="n">
-        <v>0</v>
-      </c>
-      <c r="AJ8" t="n">
-        <v>0</v>
-      </c>
-      <c r="AK8" t="n">
-        <v>0</v>
-      </c>
-      <c r="AL8" t="n">
-        <v>0</v>
-      </c>
-      <c r="AM8" t="n">
-        <v>0</v>
-      </c>
-      <c r="AN8" t="n">
-        <v>0</v>
-      </c>
-      <c r="AO8" t="n">
-        <v>0</v>
-      </c>
-      <c r="AP8" t="inlineStr"/>
-      <c r="AQ8" t="n">
-        <v>1</v>
-      </c>
-      <c r="AR8" t="n">
-        <v>1</v>
-      </c>
-      <c r="AS8" t="inlineStr"/>
-    </row>
-    <row r="9">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>nearest_neighbor_k3</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>Nearest-neighbor prediction k=3</t>
-        </is>
-      </c>
-      <c r="C9" t="n">
-        <v>17</v>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>Shower</t>
-        </is>
-      </c>
-      <c r="E9" t="n">
-        <v>17</v>
-      </c>
-      <c r="F9" t="n">
-        <v>17</v>
-      </c>
-      <c r="G9" t="inlineStr">
-        <is>
-          <t>How long should I shower?</t>
-        </is>
-      </c>
-      <c r="H9" t="inlineStr">
-        <is>
-          <t>West Mifflin, PA</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>similarity</t>
-        </is>
-      </c>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>sentence-transformers/all-MiniLM-L6-v2</t>
-        </is>
-      </c>
-      <c r="K9" t="n">
-        <v>3</v>
-      </c>
-      <c r="L9" t="b">
-        <v>1</v>
-      </c>
-      <c r="M9" t="b">
-        <v>1</v>
-      </c>
-      <c r="N9" t="b">
-        <v>1</v>
-      </c>
-      <c r="O9" t="b">
-        <v>0</v>
-      </c>
-      <c r="P9" t="inlineStr">
-        <is>
-          <t>5</t>
-        </is>
-      </c>
-      <c r="Q9" t="n">
-        <v>8.044444444444444</v>
-      </c>
-      <c r="R9" t="n">
-        <v>7.506666666666667</v>
-      </c>
-      <c r="S9" t="n">
-        <v>7.517777777777777</v>
-      </c>
-      <c r="T9" t="n">
-        <v>3.522222222222222</v>
-      </c>
-      <c r="U9" t="n">
-        <v>7.072555555555555</v>
-      </c>
-      <c r="V9" t="n">
-        <v>2</v>
-      </c>
-      <c r="W9" t="n">
-        <v>7.3695</v>
-      </c>
-      <c r="X9" t="n">
-        <v>2</v>
-      </c>
-      <c r="Y9" t="n">
-        <v>0.04096141892174879</v>
-      </c>
-      <c r="Z9" t="n">
-        <v>3</v>
-      </c>
-      <c r="AA9" t="n">
-        <v>0.3688148148148149</v>
-      </c>
-      <c r="AB9" t="n">
-        <v>0.3875168733881066</v>
-      </c>
-      <c r="AC9" t="inlineStr"/>
-      <c r="AD9" t="inlineStr"/>
-      <c r="AE9" t="b">
-        <v>1</v>
-      </c>
-      <c r="AF9" t="b">
-        <v>1</v>
-      </c>
-      <c r="AG9" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="AH9" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="AI9" t="n">
-        <v>0</v>
-      </c>
-      <c r="AJ9" t="n">
-        <v>0</v>
-      </c>
-      <c r="AK9" t="n">
-        <v>0</v>
-      </c>
-      <c r="AL9" t="n">
-        <v>0</v>
-      </c>
-      <c r="AM9" t="n">
-        <v>0</v>
-      </c>
-      <c r="AN9" t="n">
-        <v>0</v>
-      </c>
-      <c r="AO9" t="n">
-        <v>0</v>
-      </c>
-      <c r="AP9" t="inlineStr"/>
-      <c r="AQ9" t="n">
-        <v>1</v>
-      </c>
-      <c r="AR9" t="n">
-        <v>1</v>
-      </c>
-      <c r="AS9" t="inlineStr"/>
-    </row>
-    <row r="10">
-      <c r="A10" t="inlineStr">
-        <is>
-          <t>nearest_neighbor_k3</t>
-        </is>
-      </c>
-      <c r="B10" t="inlineStr">
-        <is>
-          <t>Nearest-neighbor prediction k=3</t>
-        </is>
-      </c>
-      <c r="C10" t="n">
-        <v>17</v>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>Shower</t>
-        </is>
-      </c>
-      <c r="E10" t="n">
-        <v>17</v>
-      </c>
-      <c r="F10" t="n">
-        <v>17</v>
-      </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>How long should I shower?</t>
-        </is>
-      </c>
-      <c r="H10" t="inlineStr">
-        <is>
-          <t>West Mifflin, PA</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>similarity</t>
-        </is>
-      </c>
-      <c r="J10" t="inlineStr">
-        <is>
-          <t>sentence-transformers/all-MiniLM-L6-v2</t>
-        </is>
-      </c>
-      <c r="K10" t="n">
-        <v>3</v>
-      </c>
-      <c r="L10" t="b">
-        <v>1</v>
-      </c>
-      <c r="M10" t="b">
-        <v>1</v>
-      </c>
-      <c r="N10" t="b">
-        <v>1</v>
-      </c>
-      <c r="O10" t="b">
-        <v>0</v>
-      </c>
-      <c r="P10" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
-      <c r="Q10" t="n">
-        <v>8.044444444444444</v>
-      </c>
-      <c r="R10" t="n">
-        <v>7.506666666666667</v>
-      </c>
-      <c r="S10" t="n">
-        <v>7.517777777777777</v>
-      </c>
-      <c r="T10" t="n">
-        <v>3.522222222222222</v>
-      </c>
-      <c r="U10" t="n">
-        <v>7.072555555555555</v>
-      </c>
-      <c r="V10" t="n">
-        <v>3</v>
-      </c>
-      <c r="W10" t="n">
-        <v>6.7995</v>
-      </c>
-      <c r="X10" t="n">
-        <v>3</v>
-      </c>
-      <c r="Y10" t="n">
-        <v>0.04096141892174879</v>
-      </c>
-      <c r="Z10" t="n">
-        <v>3</v>
-      </c>
-      <c r="AA10" t="n">
-        <v>0.3688148148148149</v>
-      </c>
-      <c r="AB10" t="n">
-        <v>0.3875168733881066</v>
-      </c>
-      <c r="AC10" t="inlineStr"/>
-      <c r="AD10" t="inlineStr"/>
-      <c r="AE10" t="b">
-        <v>1</v>
-      </c>
-      <c r="AF10" t="b">
-        <v>1</v>
-      </c>
-      <c r="AG10" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="AH10" t="inlineStr">
-        <is>
-          <t>3</t>
-        </is>
-      </c>
-      <c r="AI10" t="n">
-        <v>0</v>
-      </c>
-      <c r="AJ10" t="n">
-        <v>0</v>
-      </c>
-      <c r="AK10" t="n">
-        <v>0</v>
-      </c>
-      <c r="AL10" t="n">
-        <v>0</v>
-      </c>
-      <c r="AM10" t="n">
-        <v>0</v>
-      </c>
-      <c r="AN10" t="n">
-        <v>0</v>
-      </c>
-      <c r="AO10" t="n">
-        <v>0</v>
-      </c>
-      <c r="AP10" t="inlineStr"/>
-      <c r="AQ10" t="n">
-        <v>1</v>
-      </c>
-      <c r="AR10" t="n">
-        <v>1</v>
-      </c>
-      <c r="AS10" t="inlineStr"/>
+      <c r="AS7" t="n">
+        <v>1</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>